<commit_message>
BWI sync — 2026-07-20 11:53 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Albania.xlsx
+++ b/BWI/bestwine_output/bestwine_Albania.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA40"/>
+  <dimension ref="A1:AA41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4594,6 +4594,75 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Deny Liquor</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>Deny Liquor</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>80243</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="inlineStr">
+        <is>
+          <t>Tirana</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>Central Albania</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>Rruga Vaso Pasha</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>https://denyliquor.al</t>
+        </is>
+      </c>
+      <c r="J41" s="2" t="inlineStr"/>
+      <c r="K41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr"/>
+      <c r="M41" s="2" t="inlineStr"/>
+      <c r="N41" s="2" t="inlineStr">
+        <is>
+          <t>liquorsdeny@gmail.com</t>
+        </is>
+      </c>
+      <c r="O41" s="2" t="inlineStr"/>
+      <c r="P41" s="2" t="inlineStr"/>
+      <c r="Q41" s="2" t="inlineStr"/>
+      <c r="R41" s="2" t="inlineStr"/>
+      <c r="S41" s="2" t="inlineStr"/>
+      <c r="T41" s="2" t="inlineStr">
+        <is>
+          <t>https://www.instagram.com/denyliquor</t>
+        </is>
+      </c>
+      <c r="U41" s="2" t="inlineStr"/>
+      <c r="V41" s="2" t="inlineStr"/>
+      <c r="W41" s="2" t="inlineStr"/>
+      <c r="X41" s="2" t="inlineStr"/>
+      <c r="Y41" s="2" t="inlineStr"/>
+      <c r="Z41" s="2" t="inlineStr"/>
+      <c r="AA41" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
BWI sync — 2026-07-27 12:20 UTC
</commit_message>
<xml_diff>
--- a/BWI/bestwine_output/bestwine_Albania.xlsx
+++ b/BWI/bestwine_output/bestwine_Albania.xlsx
@@ -447,7 +447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA41"/>
+  <dimension ref="A1:AA42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4663,6 +4663,75 @@
       <c r="Z41" s="2" t="inlineStr"/>
       <c r="AA41" s="2" t="inlineStr"/>
     </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Eurolab Internacional Grup sh.p.k.</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr"/>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>168073</t>
+        </is>
+      </c>
+      <c r="D42" s="2" t="inlineStr">
+        <is>
+          <t>Albania</t>
+        </is>
+      </c>
+      <c r="E42" s="2" t="inlineStr">
+        <is>
+          <t>Kashar</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr"/>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Rr. Jashar Skenderi</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>1050</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.eurolabinternacional.com</t>
+        </is>
+      </c>
+      <c r="J42" s="2" t="inlineStr"/>
+      <c r="K42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr"/>
+      <c r="M42" s="2" t="inlineStr"/>
+      <c r="N42" s="2" t="inlineStr">
+        <is>
+          <t>info@eurolabinternacional.com</t>
+        </is>
+      </c>
+      <c r="O42" s="2" t="inlineStr">
+        <is>
+          <t>+355 4 453 3100</t>
+        </is>
+      </c>
+      <c r="P42" s="2" t="inlineStr"/>
+      <c r="Q42" s="2" t="inlineStr"/>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>https://www.linkedin.com/company/eurolab-internacional-grup/</t>
+        </is>
+      </c>
+      <c r="S42" s="2" t="inlineStr"/>
+      <c r="T42" s="2" t="inlineStr"/>
+      <c r="U42" s="2" t="inlineStr"/>
+      <c r="V42" s="2" t="inlineStr"/>
+      <c r="W42" s="2" t="inlineStr"/>
+      <c r="X42" s="2" t="inlineStr"/>
+      <c r="Y42" s="2" t="inlineStr"/>
+      <c r="Z42" s="2" t="inlineStr"/>
+      <c r="AA42" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>